<commit_message>
HVAC batch 1: the missed flame-sensor correction in brief #14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LAzRbJbAp9yiiRdLp2y8mb
</commit_message>
<xml_diff>
--- a/studies/hvac/ideation/batch1-briefs-2026-10-27-corrected.xlsx
+++ b/studies/hvac/ideation/batch1-briefs-2026-10-27-corrected.xlsx
@@ -680,7 +680,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>The part is the flame sensor: a thin metal rod in the burner flame that proves to the control board the gas lit. When it's coated with carbon or oxide, the board can't read the flame, so the furnace lights, runs a few seconds, shuts the gas off and retries, sometimes locking out after three tries. A new sensor costs about $10-$25; a service call to clean or replace it typically runs $100-$250, $300 or more after hours. The fix: turn off power at the furnace switch and turn the gas valve off (and let it cool), remove the burner door, take out the one screw holding the sensor, pull it out by its base, polish the rod lightly with a Scotch-Brite pad or very fine emery cloth (not coarse sandpaper; keep grit off the ceramic), wipe it, reinstall, restore power and watch a full cycle. If it still shuts off, other causes: a dirty filter (high limit), a clogged condensate trap or vent pipe (pressure switch), a weak igniter, or a bad sensor wire; that's when to call a tech. Safety: never touch the hot-surface igniter next to it (fragile, skin oils crack it); if you smell gas, stop and call the gas company. Prices as rounded ranges.</t>
+          <t>The part is the flame sensor: a thin metal rod in the burner flame that proves to the control board the gas lit. When it's coated with carbon or oxide, the board can't read the flame, so the furnace lights, runs a few seconds, shuts the gas off and retries, sometimes locking out after three tries. A new sensor costs about $10-$30; a service call to clean or replace it typically runs $100-$250, up to about $300 at night or on a weekend. The fix: turn off power at the furnace switch and turn the gas valve off (and let it cool), remove the burner door, take out the one screw holding the sensor, pull it out by its base, polish the rod lightly with a Scotch-Brite pad or very fine emery cloth (not coarse sandpaper; keep grit off the ceramic), wipe it, reinstall, restore power and watch a full cycle. If it still shuts off, other causes: a dirty filter (high limit), a clogged condensate trap or vent pipe (pressure switch), a weak igniter, or a bad sensor wire; that's when to call a tech. Safety: never touch the hot-surface igniter next to it (fragile, skin oils crack it); if you smell gas, stop and call the gas company. Prices as rounded ranges.</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1493,51 +1493,51 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>You've Been Running Your Ceiling Fan WRONG All Winter — Flip This Switch Tonight</t>
+          <t>Furnace Keeps Shutting Off? The $12 Part Techs Charge $300 to Replace (Clean It Yourself)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>(the DOE's setback figure works out to roughly 1% a year per degree for 8 hours a day; keep the claim soft, never 'cuts your bill')</t>
+          <t>A new sensor costs about $10-$25; a service call to clean or replace it typically runs $100-$250, $300 or more after hours.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>(the DOE's heating and cooling guide says about 1% off the heating bill for each degree set back for eight hours; 'a degree or two lower' itself isn't DOE wording, so it's said in words; keep the claim soft, never 'cuts your bill')</t>
+          <t>A new sensor costs about $10-$30; a service call to clean or replace it typically runs $100-$250, up to about $300 at night or on a weekend.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>D-verify: the 1% figure is on a live DOE file (2021), for the heating bill, not 'a year'; the fan line stays in words</t>
+          <t>A-research flag ('$300' is the top, not typical: say 'up to $300') and A-verify (part $10-$30); added 2026-10-27 after it was missed in the first pass</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Why Buy a Generator? Your Car Can Keep Your Furnace Running in an Outage</t>
+          <t>You've Been Running Your Ceiling Fan WRONG All Winter — Flip This Switch Tonight</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>but it only needs about 300-800 watts</t>
+          <t>(the DOE's setback figure works out to roughly 1% a year per degree for 8 hours a day; keep the claim soft, never 'cuts your bill')</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>but it only needs about 400-800 watts to run, with a start-up surge that can reach 1,400 or more on an older blower motor</t>
+          <t>(the DOE's heating and cooling guide says about 1% off the heating bill for each degree set back for eight hours; 'a degree or two lower' itself isn't DOE wording, so it's said in words; keep the claim soft, never 'cuts your bill')</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>D-research and D-verify (in words; check the blower's label)</t>
+          <t>D-verify: the 1% figure is on a live DOE file (2021), for the heating bill, not 'a year'; the fan line stays in words</t>
         </is>
       </c>
     </row>
@@ -1552,17 +1552,17 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>(about $100-$250 for a 1,000-1,500 watt model)</t>
+          <t>but it only needs about 300-800 watts</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>(about $150-$300 for a decent 1,000-1,500 watt pure sine model)</t>
+          <t>but it only needs about 400-800 watts to run, with a start-up surge that can reach 1,400 or more on an older blower motor</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>C-verify: pure sine $150-$300; the $90-$130 ones are modified sine</t>
+          <t>D-research and D-verify (in words; check the blower's label)</t>
         </is>
       </c>
     </row>
@@ -1577,17 +1577,17 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>(often $200-$500)</t>
+          <t>(about $100-$250 for a 1,000-1,500 watt model)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>(the switch is about $100-$150, plus a few hundred dollars for the electrician; no checked installed figure)</t>
+          <t>(about $150-$300 for a decent 1,000-1,500 watt pure sine model)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>C-research and C-verify: '$200-$500 installed' not confirmed; in words</t>
+          <t>C-verify: pure sine $150-$300; the $90-$130 ones are modified sine</t>
         </is>
       </c>
     </row>
@@ -1602,15 +1602,40 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
+          <t>(often $200-$500)</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>(the switch is about $100-$150, plus a few hundred dollars for the electrician; no checked installed figure)</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>C-research and C-verify: '$200-$500 installed' not confirmed; in words</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Why Buy a Generator? Your Car Can Keep Your Furnace Running in an Outage</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
           <t>at least 20 feet from doors, windows and vents (CPSC's distance for generators)</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>well away from the house (20 feet from doors, windows and vents is the CPSC and CDC distance for generators; there's no official distance for a car, so the script says it in words)</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>D-research flag 2: 20 feet is the generator distance; no official car distance</t>
         </is>

</xml_diff>